<commit_message>
created a Vercel prisma db, updated Project-status.md
</commit_message>
<xml_diff>
--- a/public/dishes-raw/millewee boissons.xlsx
+++ b/public/dishes-raw/millewee boissons.xlsx
@@ -1,12 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sorin\Documents\GitHub\innopay-full\millewee\public\dishes-raw\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23235" windowHeight="9630"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Extraction des Boissons et Vins" sheetId="1" r:id="rId5"/>
+    <sheet name="millewee boissons" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -388,21 +396,23 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -413,43 +423,44 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -639,25 +650,28 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="15.0"/>
-    <col customWidth="1" min="2" max="2" width="26.88"/>
-    <col customWidth="1" min="3" max="3" width="44.38"/>
-    <col customWidth="1" min="4" max="4" width="23.75"/>
-    <col customWidth="1" min="5" max="5" width="20.88"/>
-    <col customWidth="1" min="6" max="6" width="27.38"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="44.42578125" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" customWidth="1"/>
+    <col min="6" max="6" width="27.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -677,7 +691,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -692,7 +706,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -707,7 +721,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -722,7 +736,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -737,7 +751,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -752,7 +766,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -767,7 +781,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -784,7 +798,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -801,7 +815,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -816,7 +830,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
@@ -831,7 +845,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>32</v>
       </c>
@@ -846,7 +860,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>32</v>
       </c>
@@ -861,7 +875,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
@@ -876,7 +890,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
@@ -889,7 +903,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
@@ -902,7 +916,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -915,7 +929,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>46</v>
       </c>
@@ -930,7 +944,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>46</v>
       </c>
@@ -945,7 +959,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>46</v>
       </c>
@@ -960,7 +974,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>55</v>
       </c>
@@ -975,7 +989,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>55</v>
       </c>
@@ -990,7 +1004,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>55</v>
       </c>
@@ -1005,7 +1019,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>55</v>
       </c>
@@ -1020,7 +1034,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>55</v>
       </c>
@@ -1035,7 +1049,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>69</v>
       </c>
@@ -1050,7 +1064,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>69</v>
       </c>
@@ -1064,7 +1078,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>69</v>
       </c>
@@ -1081,7 +1095,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>79</v>
       </c>
@@ -1096,7 +1110,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>79</v>
       </c>
@@ -1111,7 +1125,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>79</v>
       </c>
@@ -1124,7 +1138,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>79</v>
       </c>
@@ -1137,7 +1151,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>85</v>
       </c>
@@ -1152,7 +1166,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>85</v>
       </c>
@@ -1164,7 +1178,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>87</v>
       </c>
@@ -1178,7 +1192,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>91</v>
       </c>
@@ -1195,7 +1209,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>91</v>
       </c>
@@ -1212,7 +1226,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>91</v>
       </c>
@@ -1229,7 +1243,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>101</v>
       </c>
@@ -1246,7 +1260,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>101</v>
       </c>
@@ -1263,7 +1277,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>107</v>
       </c>
@@ -1280,7 +1294,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>107</v>
       </c>
@@ -1297,7 +1311,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>107</v>
       </c>
@@ -1314,7 +1328,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>107</v>
       </c>
@@ -1331,7 +1345,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>118</v>
       </c>
@@ -1345,7 +1359,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>118</v>
       </c>
@@ -1360,6 +1374,6 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>